<commit_message>
Refactor: remove underpowered Clove group from Bay Leaf Assay
</commit_message>
<xml_diff>
--- a/cleaning/OXIDATIVE_STRESS_MARKERS_CONSOLIDATED.xlsx
+++ b/cleaning/OXIDATIVE_STRESS_MARKERS_CONSOLIDATED.xlsx
@@ -1785,7 +1785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.140625" customWidth="1" min="1" max="1"/>
@@ -2790,294 +2790,168 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>CL (Clove Extract - CL 16-17)</t>
+          <t>p-value (MG vs NG)</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>1.1504 ± 0.2566</t>
+          <t>0.9866 (ns)</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>1.6703 ± 0.3716</t>
+          <t>0.9887 (ns)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>0.5725 ± 0.0648</t>
+          <t>0.8443 (ns)</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>1.7265 ± 0.3234</t>
+          <t>0.9821 (ns)</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>0.2082 ± 0.0565</t>
+          <t>0.9998 (ns)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>69.1803 ± 0.9836</t>
+          <t>0.9985 (ns)</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>20.4797 ± 5.2768</t>
+          <t>0.9535 (ns)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>p-value (MG vs NG)</t>
+          <t>p-value (BL vs MG)</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>0.9971 (ns)</t>
+          <t>0.6331 (ns)</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>0.9979 (ns)</t>
+          <t>0.8388 (ns)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>0.9165 (ns)</t>
+          <t>0.8275 (ns)</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>0.9957 (ns)</t>
+          <t>0.2866 (ns)</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>1.0000 (ns)</t>
+          <t>0.5489 (ns)</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>0.9998 (ns)</t>
+          <t>0.9923 (ns)</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>0.9873 (ns)</t>
+          <t>0.9909 (ns)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>p-value (BL vs MG)</t>
+          <t>p-value (IBU vs MG)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>0.7548 (ns)</t>
+          <t>0.9812 (ns)</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>0.9243 (ns)</t>
+          <t>0.9953 (ns)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>0.9043 (ns)</t>
+          <t>0.7176 (ns)</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>0.3864 (ns)</t>
+          <t>0.5403 (ns)</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>0.6683 (ns)</t>
+          <t>0.9199 (ns)</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>0.9985 (ns)</t>
+          <t>1.0000 (ns)</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>0.9986 (ns)</t>
+          <t>0.9991 (ns)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>p-value (IBU vs MG)</t>
+          <t>p-value (BL vs IBU)</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>0.9955 (ns)</t>
+          <t>0.8903 (ns)</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>0.9993 (ns)</t>
+          <t>0.9512 (ns)</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>0.8153 (ns)</t>
+          <t>0.9553 (ns)</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>0.6660 (ns)</t>
+          <t>0.9998 (ns)</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>0.9676 (ns)</t>
+          <t>0.9526 (ns)</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>1.0000 (ns)</t>
+          <t>0.9905 (ns)</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>0.9999 (ns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>p-value (CL vs MG)</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>0.9186 (ns)</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>0.9308 (ns)</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>0.9511 (ns)</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>0.5611 (ns)</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>0.9998 (ns)</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>1.0000 (ns)</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>0.9027 (ns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>p-value (BL vs IBU)</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>0.9519 (ns)</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>0.9849 (ns)</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>0.9842 (ns)</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>1.0000 (ns)</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>0.9839 (ns)</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>0.9980 (ns)</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>0.9914 (ns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>p-value (CL vs IBU)</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>0.9871 (ns)</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>0.9759 (ns)</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>0.9990 (ns)</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>0.9977 (ns)</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>0.9947 (ns)</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>1.0000 (ns)</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>0.8568 (ns)</t>
+          <t>0.9651 (ns)</t>
         </is>
       </c>
     </row>

</xml_diff>